<commit_message>
Add current SCEDULAR changes
</commit_message>
<xml_diff>
--- a/SCEDULAR_SEM3_SHORTCUT_INPUT.xlsx
+++ b/SCEDULAR_SEM3_SHORTCUT_INPUT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f6a4d0bb458c816a/Desktop/TIME_TABLE_SCHEDULAR/New folder/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f6a4d0bb458c816a/Desktop/TIME_TABLE_SCHEDULAR/SCEDULAR/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="12" documentId="11_0ED6138A4E78080133F7CB7D9D22B29320E93D2E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AC11FCF-D68F-48A8-9390-01DB422F8108}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1080" yWindow="1080" windowWidth="17280" windowHeight="9960" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>

</xml_diff>